<commit_message>
Wrote some of the final paper
</commit_message>
<xml_diff>
--- a/binary-search/PerformanceData/binarySearchPerformanceData.xlsx
+++ b/binary-search/PerformanceData/binarySearchPerformanceData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark Stotzer\Documents\Mark\CSC360\csc360-project\binary-search\PerformanceData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark Stotzer\Documents\Mark\CSC360\csc360Current\binary-search\PerformanceData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1746642-1E8F-47EB-83A2-0195FECD886D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{804BFA0F-8E58-4C28-9966-0B600F3010BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -83,16 +83,10 @@
     <t>Compiler Algorithm</t>
   </si>
   <si>
-    <t>Handwritten Algorithm</t>
-  </si>
-  <si>
     <t>Single-Stage</t>
   </si>
   <si>
     <t>5-Stage</t>
-  </si>
-  <si>
-    <t>Handwritten</t>
   </si>
   <si>
     <t>Naïve</t>
@@ -102,6 +96,12 @@
   </si>
   <si>
     <t>Clock Cycles</t>
+  </si>
+  <si>
+    <t>Best Algorithm</t>
+  </si>
+  <si>
+    <t>Best</t>
   </si>
 </sst>
 </file>
@@ -553,21 +553,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -585,6 +570,21 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -819,7 +819,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Handwritten</c:v>
+                  <c:v>Best</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1492,7 +1492,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Handwritten</c:v>
+                  <c:v>Best</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3407,21 +3407,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="27"/>
-      <c r="J1" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
+      <c r="A1" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="31"/>
+      <c r="J1" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1" s="32"/>
+      <c r="L1" s="32"/>
+      <c r="M1" s="32"/>
     </row>
     <row r="2" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="14" t="s">
@@ -3447,13 +3447,13 @@
       </c>
       <c r="J2" s="20"/>
       <c r="K2" s="20" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L2" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="M2" s="20" t="s">
         <v>18</v>
-      </c>
-      <c r="M2" s="20" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
@@ -3473,7 +3473,7 @@
         <f>D3/C3</f>
         <v>1</v>
       </c>
-      <c r="F3" s="31">
+      <c r="F3" s="26">
         <v>30</v>
       </c>
       <c r="G3" s="13">
@@ -3481,7 +3481,7 @@
         <v>1.8</v>
       </c>
       <c r="J3" s="20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K3" s="19">
         <f>C17</f>
@@ -3511,13 +3511,13 @@
         <f t="shared" ref="E4:E5" si="0">D4/C4</f>
         <v>1</v>
       </c>
-      <c r="F4" s="32"/>
+      <c r="F4" s="27"/>
       <c r="G4" s="13">
         <f t="shared" ref="G4:G6" si="1">C4/$F$3</f>
         <v>1.4666666666666666</v>
       </c>
       <c r="J4" s="21" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K4" s="22">
         <f>C21</f>
@@ -3547,17 +3547,17 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="F5" s="32"/>
+      <c r="F5" s="27"/>
       <c r="G5" s="13">
         <f t="shared" si="1"/>
         <v>1.6666666666666667</v>
       </c>
-      <c r="J5" s="24" t="s">
+      <c r="J5" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="K5" s="24"/>
-      <c r="L5" s="24"/>
-      <c r="M5" s="24"/>
+      <c r="K5" s="33"/>
+      <c r="L5" s="33"/>
+      <c r="M5" s="33"/>
     </row>
     <row r="6" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="36"/>
@@ -3576,20 +3576,20 @@
         <f>D6/C6</f>
         <v>1</v>
       </c>
-      <c r="F6" s="33"/>
+      <c r="F6" s="28"/>
       <c r="G6" s="13">
         <f t="shared" si="1"/>
         <v>1.6444444444444446</v>
       </c>
       <c r="J6" s="20"/>
       <c r="K6" s="20" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L6" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="M6" s="20" t="s">
         <v>18</v>
-      </c>
-      <c r="M6" s="20" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
@@ -3609,7 +3609,7 @@
         <f>D7/C7</f>
         <v>0.69230769230769229</v>
       </c>
-      <c r="F7" s="31">
+      <c r="F7" s="26">
         <v>115</v>
       </c>
       <c r="G7" s="13">
@@ -3617,7 +3617,7 @@
         <v>0.67826086956521736</v>
       </c>
       <c r="J7" s="20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K7" s="19">
         <f>G17</f>
@@ -3647,13 +3647,13 @@
         <f>D8/C8</f>
         <v>0.61971830985915488</v>
       </c>
-      <c r="F8" s="32"/>
+      <c r="F8" s="27"/>
       <c r="G8" s="13">
         <f t="shared" ref="G8:G10" si="2">C8/$F$7</f>
         <v>0.61739130434782608</v>
       </c>
       <c r="J8" s="20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K8" s="19">
         <f>G21</f>
@@ -3683,7 +3683,7 @@
         <f>D9/C9</f>
         <v>0.67567567567567566</v>
       </c>
-      <c r="F9" s="32"/>
+      <c r="F9" s="27"/>
       <c r="G9" s="13">
         <f t="shared" si="2"/>
         <v>0.64347826086956517</v>
@@ -3706,7 +3706,7 @@
         <f>D10/C10</f>
         <v>0.66367713004484308</v>
       </c>
-      <c r="F10" s="33"/>
+      <c r="F10" s="28"/>
       <c r="G10" s="13">
         <f t="shared" si="2"/>
         <v>0.6463768115942029</v>
@@ -3714,15 +3714,15 @@
     </row>
     <row r="11" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="12" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="25" t="s">
+      <c r="A12" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="27"/>
+      <c r="B12" s="30"/>
+      <c r="C12" s="30"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="30"/>
+      <c r="F12" s="30"/>
+      <c r="G12" s="31"/>
     </row>
     <row r="13" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
@@ -3748,7 +3748,7 @@
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A14" s="28" t="s">
+      <c r="A14" s="23" t="s">
         <v>4</v>
       </c>
       <c r="B14" s="9" t="s">
@@ -3764,7 +3764,7 @@
         <f t="shared" ref="E14:E21" si="3">D14/C14</f>
         <v>1</v>
       </c>
-      <c r="F14" s="31">
+      <c r="F14" s="26">
         <v>30</v>
       </c>
       <c r="G14" s="13">
@@ -3773,7 +3773,7 @@
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A15" s="29"/>
+      <c r="A15" s="24"/>
       <c r="B15" s="10" t="s">
         <v>6</v>
       </c>
@@ -3787,14 +3787,14 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F15" s="32"/>
+      <c r="F15" s="27"/>
       <c r="G15" s="13">
         <f t="shared" ref="G15:G17" si="4">C15/$F$14</f>
         <v>1.4666666666666666</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A16" s="29"/>
+      <c r="A16" s="24"/>
       <c r="B16" s="10" t="s">
         <v>7</v>
       </c>
@@ -3808,14 +3808,14 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F16" s="32"/>
+      <c r="F16" s="27"/>
       <c r="G16" s="13">
         <f t="shared" si="4"/>
         <v>1.6666666666666667</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="30"/>
+      <c r="A17" s="25"/>
       <c r="B17" s="11" t="s">
         <v>8</v>
       </c>
@@ -3831,14 +3831,14 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F17" s="33"/>
+      <c r="F17" s="28"/>
       <c r="G17" s="13">
         <f t="shared" si="4"/>
         <v>1.6444444444444446</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="28" t="s">
+      <c r="A18" s="23" t="s">
         <v>0</v>
       </c>
       <c r="B18" s="12" t="s">
@@ -3854,7 +3854,7 @@
         <f t="shared" si="3"/>
         <v>0.62790697674418605</v>
       </c>
-      <c r="F18" s="31">
+      <c r="F18" s="26">
         <v>115</v>
       </c>
       <c r="G18" s="13">
@@ -3863,7 +3863,7 @@
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="29"/>
+      <c r="A19" s="24"/>
       <c r="B19" s="10" t="s">
         <v>6</v>
       </c>
@@ -3877,14 +3877,14 @@
         <f t="shared" si="3"/>
         <v>0.5714285714285714</v>
       </c>
-      <c r="F19" s="32"/>
+      <c r="F19" s="27"/>
       <c r="G19" s="13">
         <f t="shared" ref="G19:G21" si="5">C19/$F$18</f>
         <v>0.66956521739130437</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="29"/>
+      <c r="A20" s="24"/>
       <c r="B20" s="10" t="s">
         <v>7</v>
       </c>
@@ -3898,14 +3898,14 @@
         <f t="shared" si="3"/>
         <v>0.64102564102564108</v>
       </c>
-      <c r="F20" s="32"/>
+      <c r="F20" s="27"/>
       <c r="G20" s="13">
         <f t="shared" si="5"/>
         <v>0.67826086956521736</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="30"/>
+      <c r="A21" s="25"/>
       <c r="B21" s="11" t="s">
         <v>8</v>
       </c>
@@ -3921,7 +3921,7 @@
         <f t="shared" si="3"/>
         <v>0.61410788381742742</v>
       </c>
-      <c r="F21" s="33"/>
+      <c r="F21" s="28"/>
       <c r="G21" s="13">
         <f t="shared" si="5"/>
         <v>0.69855072463768109</v>
@@ -3929,15 +3929,15 @@
     </row>
     <row r="22" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="23" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="25" t="s">
+      <c r="A23" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="B23" s="26"/>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="26"/>
-      <c r="F23" s="26"/>
-      <c r="G23" s="27"/>
+      <c r="B23" s="30"/>
+      <c r="C23" s="30"/>
+      <c r="D23" s="30"/>
+      <c r="E23" s="30"/>
+      <c r="F23" s="30"/>
+      <c r="G23" s="31"/>
     </row>
     <row r="24" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="14" t="s">
@@ -3963,7 +3963,7 @@
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="28" t="s">
+      <c r="A25" s="23" t="s">
         <v>4</v>
       </c>
       <c r="B25" s="9" t="s">
@@ -3979,7 +3979,7 @@
         <f t="shared" ref="E25:E32" si="6">D25/C25</f>
         <v>1</v>
       </c>
-      <c r="F25" s="31">
+      <c r="F25" s="26">
         <v>30</v>
       </c>
       <c r="G25" s="13">
@@ -3988,7 +3988,7 @@
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" s="29"/>
+      <c r="A26" s="24"/>
       <c r="B26" s="10" t="s">
         <v>6</v>
       </c>
@@ -4002,14 +4002,14 @@
         <f t="shared" si="6"/>
         <v>1</v>
       </c>
-      <c r="F26" s="32"/>
+      <c r="F26" s="27"/>
       <c r="G26" s="13">
         <f t="shared" ref="G26:G28" si="7">C26/$F$25</f>
         <v>1.5333333333333334</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="29"/>
+      <c r="A27" s="24"/>
       <c r="B27" s="10" t="s">
         <v>7</v>
       </c>
@@ -4023,14 +4023,14 @@
         <f t="shared" si="6"/>
         <v>1</v>
       </c>
-      <c r="F27" s="32"/>
+      <c r="F27" s="27"/>
       <c r="G27" s="13">
         <f t="shared" si="7"/>
         <v>1.7666666666666666</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="30"/>
+      <c r="A28" s="25"/>
       <c r="B28" s="11" t="s">
         <v>8</v>
       </c>
@@ -4046,14 +4046,14 @@
         <f t="shared" si="6"/>
         <v>1</v>
       </c>
-      <c r="F28" s="33"/>
+      <c r="F28" s="28"/>
       <c r="G28" s="13">
         <f t="shared" si="7"/>
         <v>1.7222222222222221</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A29" s="28" t="s">
+      <c r="A29" s="23" t="s">
         <v>0</v>
       </c>
       <c r="B29" s="12" t="s">
@@ -4069,7 +4069,7 @@
         <f t="shared" si="6"/>
         <v>0.7</v>
       </c>
-      <c r="F29" s="31">
+      <c r="F29" s="26">
         <v>115</v>
       </c>
       <c r="G29" s="13">
@@ -4078,7 +4078,7 @@
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A30" s="29"/>
+      <c r="A30" s="24"/>
       <c r="B30" s="10" t="s">
         <v>6</v>
       </c>
@@ -4092,14 +4092,14 @@
         <f t="shared" si="6"/>
         <v>0.63013698630136983</v>
       </c>
-      <c r="F30" s="32"/>
+      <c r="F30" s="27"/>
       <c r="G30" s="13">
         <f t="shared" ref="G30:G32" si="8">C30/$F$29</f>
         <v>0.63478260869565217</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A31" s="29"/>
+      <c r="A31" s="24"/>
       <c r="B31" s="10" t="s">
         <v>7</v>
       </c>
@@ -4113,14 +4113,14 @@
         <f t="shared" si="6"/>
         <v>0.68831168831168832</v>
       </c>
-      <c r="F31" s="32"/>
+      <c r="F31" s="27"/>
       <c r="G31" s="13">
         <f t="shared" si="8"/>
         <v>0.66956521739130437</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="30"/>
+      <c r="A32" s="25"/>
       <c r="B32" s="11" t="s">
         <v>8</v>
       </c>
@@ -4136,7 +4136,7 @@
         <f t="shared" si="6"/>
         <v>0.67391304347826075</v>
       </c>
-      <c r="F32" s="33"/>
+      <c r="F32" s="28"/>
       <c r="G32" s="13">
         <f t="shared" si="8"/>
         <v>0.66666666666666674</v>
@@ -4144,13 +4144,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A29:A32"/>
-    <mergeCell ref="F29:F32"/>
-    <mergeCell ref="A12:G12"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="F14:F17"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="F18:F21"/>
     <mergeCell ref="J1:M1"/>
     <mergeCell ref="J5:M5"/>
     <mergeCell ref="A23:G23"/>
@@ -4161,6 +4154,13 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="F7:F10"/>
     <mergeCell ref="F3:F6"/>
+    <mergeCell ref="A29:A32"/>
+    <mergeCell ref="F29:F32"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="F14:F17"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="F18:F21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Worked on binary search sections of final paper
</commit_message>
<xml_diff>
--- a/binary-search/PerformanceData/binarySearchPerformanceData.xlsx
+++ b/binary-search/PerformanceData/binarySearchPerformanceData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark Stotzer\Documents\Mark\CSC360\csc360-project\binary-search\PerformanceData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark Stotzer\Documents\Mark\CSC360\csc360Current\binary-search\PerformanceData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1746642-1E8F-47EB-83A2-0195FECD886D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16771A61-5F16-48BC-A781-7F4F6E7F26CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -83,16 +83,7 @@
     <t>Compiler Algorithm</t>
   </si>
   <si>
-    <t>Handwritten Algorithm</t>
-  </si>
-  <si>
     <t>Single-Stage</t>
-  </si>
-  <si>
-    <t>5-Stage</t>
-  </si>
-  <si>
-    <t>Handwritten</t>
   </si>
   <si>
     <t>Naïve</t>
@@ -102,6 +93,15 @@
   </si>
   <si>
     <t>Clock Cycles</t>
+  </si>
+  <si>
+    <t>Modified</t>
+  </si>
+  <si>
+    <t>Modified Algorithm</t>
+  </si>
+  <si>
+    <t>Five-Stage</t>
   </si>
 </sst>
 </file>
@@ -784,7 +784,7 @@
                   <c:v>Single-Stage</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5-Stage</c:v>
+                  <c:v>Five-Stage</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -819,7 +819,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Handwritten</c:v>
+                  <c:v>Modified</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -901,7 +901,7 @@
                   <c:v>Single-Stage</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5-Stage</c:v>
+                  <c:v>Five-Stage</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1018,7 +1018,7 @@
                   <c:v>Single-Stage</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5-Stage</c:v>
+                  <c:v>Five-Stage</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1457,7 +1457,7 @@
                   <c:v>Single-Stage</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5-Stage</c:v>
+                  <c:v>Five-Stage</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1492,7 +1492,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Handwritten</c:v>
+                  <c:v>Modified</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1574,7 +1574,7 @@
                   <c:v>Single-Stage</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5-Stage</c:v>
+                  <c:v>Five-Stage</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1691,7 +1691,7 @@
                   <c:v>Single-Stage</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5-Stage</c:v>
+                  <c:v>Five-Stage</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3408,7 +3408,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="25" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
@@ -3417,7 +3417,7 @@
       <c r="F1" s="26"/>
       <c r="G1" s="27"/>
       <c r="J1" s="23" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="K1" s="23"/>
       <c r="L1" s="23"/>
@@ -3447,13 +3447,13 @@
       </c>
       <c r="J2" s="20"/>
       <c r="K2" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="L2" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="L2" s="20" t="s">
-        <v>18</v>
-      </c>
       <c r="M2" s="20" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
@@ -3481,7 +3481,7 @@
         <v>1.8</v>
       </c>
       <c r="J3" s="20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K3" s="19">
         <f>C17</f>
@@ -3517,7 +3517,7 @@
         <v>1.4666666666666666</v>
       </c>
       <c r="J4" s="21" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="K4" s="22">
         <f>C21</f>
@@ -3583,13 +3583,13 @@
       </c>
       <c r="J6" s="20"/>
       <c r="K6" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="L6" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="L6" s="20" t="s">
-        <v>18</v>
-      </c>
       <c r="M6" s="20" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
@@ -3617,7 +3617,7 @@
         <v>0.67826086956521736</v>
       </c>
       <c r="J7" s="20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K7" s="19">
         <f>G17</f>
@@ -3632,7 +3632,7 @@
         <v>1.7222222222222221</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="35"/>
       <c r="B8" s="10" t="s">
         <v>6</v>
@@ -3652,8 +3652,8 @@
         <f t="shared" ref="G8:G10" si="2">C8/$F$7</f>
         <v>0.61739130434782608</v>
       </c>
-      <c r="J8" s="20" t="s">
-        <v>17</v>
+      <c r="J8" s="21" t="s">
+        <v>21</v>
       </c>
       <c r="K8" s="19">
         <f>G21</f>

</xml_diff>

<commit_message>
Fixed binary search charts
</commit_message>
<xml_diff>
--- a/binary-search/PerformanceData/binarySearchPerformanceData.xlsx
+++ b/binary-search/PerformanceData/binarySearchPerformanceData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark Stotzer\Documents\Mark\CSC360\csc360Current\binary-search\PerformanceData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16771A61-5F16-48BC-A781-7F4F6E7F26CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A272F6F5-948D-4197-8DEB-BEC6312454CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -553,21 +553,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -585,6 +570,21 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -647,13 +647,8 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Clock Cycles by</a:t>
+              <a:t>Binary Search Clock Cycles</a:t>
             </a:r>
-            <a:r>
-              <a:rPr lang="en-US" baseline="0"/>
-              <a:t> Algorithm</a:t>
-            </a:r>
-            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:rich>
       </c:tx>
@@ -1117,6 +1112,20 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
         <c:title>
           <c:tx>
             <c:rich>
@@ -1172,7 +1181,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1325,7 +1334,15 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Execution Time by Algorithm</a:t>
+              <a:t>Binary</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> Search </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Execution Time</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1789,6 +1806,20 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
         <c:title>
           <c:tx>
             <c:rich>
@@ -3407,21 +3438,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="27"/>
-      <c r="J1" s="23" t="s">
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="31"/>
+      <c r="J1" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
+      <c r="K1" s="32"/>
+      <c r="L1" s="32"/>
+      <c r="M1" s="32"/>
     </row>
     <row r="2" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="14" t="s">
@@ -3473,7 +3504,7 @@
         <f>D3/C3</f>
         <v>1</v>
       </c>
-      <c r="F3" s="31">
+      <c r="F3" s="26">
         <v>30</v>
       </c>
       <c r="G3" s="13">
@@ -3511,7 +3542,7 @@
         <f t="shared" ref="E4:E5" si="0">D4/C4</f>
         <v>1</v>
       </c>
-      <c r="F4" s="32"/>
+      <c r="F4" s="27"/>
       <c r="G4" s="13">
         <f t="shared" ref="G4:G6" si="1">C4/$F$3</f>
         <v>1.4666666666666666</v>
@@ -3547,17 +3578,17 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="F5" s="32"/>
+      <c r="F5" s="27"/>
       <c r="G5" s="13">
         <f t="shared" si="1"/>
         <v>1.6666666666666667</v>
       </c>
-      <c r="J5" s="24" t="s">
+      <c r="J5" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="K5" s="24"/>
-      <c r="L5" s="24"/>
-      <c r="M5" s="24"/>
+      <c r="K5" s="33"/>
+      <c r="L5" s="33"/>
+      <c r="M5" s="33"/>
     </row>
     <row r="6" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="36"/>
@@ -3576,7 +3607,7 @@
         <f>D6/C6</f>
         <v>1</v>
       </c>
-      <c r="F6" s="33"/>
+      <c r="F6" s="28"/>
       <c r="G6" s="13">
         <f t="shared" si="1"/>
         <v>1.6444444444444446</v>
@@ -3609,7 +3640,7 @@
         <f>D7/C7</f>
         <v>0.69230769230769229</v>
       </c>
-      <c r="F7" s="31">
+      <c r="F7" s="26">
         <v>115</v>
       </c>
       <c r="G7" s="13">
@@ -3647,7 +3678,7 @@
         <f>D8/C8</f>
         <v>0.61971830985915488</v>
       </c>
-      <c r="F8" s="32"/>
+      <c r="F8" s="27"/>
       <c r="G8" s="13">
         <f t="shared" ref="G8:G10" si="2">C8/$F$7</f>
         <v>0.61739130434782608</v>
@@ -3683,7 +3714,7 @@
         <f>D9/C9</f>
         <v>0.67567567567567566</v>
       </c>
-      <c r="F9" s="32"/>
+      <c r="F9" s="27"/>
       <c r="G9" s="13">
         <f t="shared" si="2"/>
         <v>0.64347826086956517</v>
@@ -3706,7 +3737,7 @@
         <f>D10/C10</f>
         <v>0.66367713004484308</v>
       </c>
-      <c r="F10" s="33"/>
+      <c r="F10" s="28"/>
       <c r="G10" s="13">
         <f t="shared" si="2"/>
         <v>0.6463768115942029</v>
@@ -3714,15 +3745,15 @@
     </row>
     <row r="11" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="12" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="25" t="s">
+      <c r="A12" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="27"/>
+      <c r="B12" s="30"/>
+      <c r="C12" s="30"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="30"/>
+      <c r="F12" s="30"/>
+      <c r="G12" s="31"/>
     </row>
     <row r="13" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
@@ -3748,7 +3779,7 @@
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A14" s="28" t="s">
+      <c r="A14" s="23" t="s">
         <v>4</v>
       </c>
       <c r="B14" s="9" t="s">
@@ -3764,7 +3795,7 @@
         <f t="shared" ref="E14:E21" si="3">D14/C14</f>
         <v>1</v>
       </c>
-      <c r="F14" s="31">
+      <c r="F14" s="26">
         <v>30</v>
       </c>
       <c r="G14" s="13">
@@ -3773,7 +3804,7 @@
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A15" s="29"/>
+      <c r="A15" s="24"/>
       <c r="B15" s="10" t="s">
         <v>6</v>
       </c>
@@ -3787,14 +3818,14 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F15" s="32"/>
+      <c r="F15" s="27"/>
       <c r="G15" s="13">
         <f t="shared" ref="G15:G17" si="4">C15/$F$14</f>
         <v>1.4666666666666666</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A16" s="29"/>
+      <c r="A16" s="24"/>
       <c r="B16" s="10" t="s">
         <v>7</v>
       </c>
@@ -3808,14 +3839,14 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F16" s="32"/>
+      <c r="F16" s="27"/>
       <c r="G16" s="13">
         <f t="shared" si="4"/>
         <v>1.6666666666666667</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="30"/>
+      <c r="A17" s="25"/>
       <c r="B17" s="11" t="s">
         <v>8</v>
       </c>
@@ -3831,14 +3862,14 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F17" s="33"/>
+      <c r="F17" s="28"/>
       <c r="G17" s="13">
         <f t="shared" si="4"/>
         <v>1.6444444444444446</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="28" t="s">
+      <c r="A18" s="23" t="s">
         <v>0</v>
       </c>
       <c r="B18" s="12" t="s">
@@ -3854,7 +3885,7 @@
         <f t="shared" si="3"/>
         <v>0.62790697674418605</v>
       </c>
-      <c r="F18" s="31">
+      <c r="F18" s="26">
         <v>115</v>
       </c>
       <c r="G18" s="13">
@@ -3863,7 +3894,7 @@
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="29"/>
+      <c r="A19" s="24"/>
       <c r="B19" s="10" t="s">
         <v>6</v>
       </c>
@@ -3877,14 +3908,14 @@
         <f t="shared" si="3"/>
         <v>0.5714285714285714</v>
       </c>
-      <c r="F19" s="32"/>
+      <c r="F19" s="27"/>
       <c r="G19" s="13">
         <f t="shared" ref="G19:G21" si="5">C19/$F$18</f>
         <v>0.66956521739130437</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="29"/>
+      <c r="A20" s="24"/>
       <c r="B20" s="10" t="s">
         <v>7</v>
       </c>
@@ -3898,14 +3929,14 @@
         <f t="shared" si="3"/>
         <v>0.64102564102564108</v>
       </c>
-      <c r="F20" s="32"/>
+      <c r="F20" s="27"/>
       <c r="G20" s="13">
         <f t="shared" si="5"/>
         <v>0.67826086956521736</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="30"/>
+      <c r="A21" s="25"/>
       <c r="B21" s="11" t="s">
         <v>8</v>
       </c>
@@ -3921,7 +3952,7 @@
         <f t="shared" si="3"/>
         <v>0.61410788381742742</v>
       </c>
-      <c r="F21" s="33"/>
+      <c r="F21" s="28"/>
       <c r="G21" s="13">
         <f t="shared" si="5"/>
         <v>0.69855072463768109</v>
@@ -3929,15 +3960,15 @@
     </row>
     <row r="22" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="23" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="25" t="s">
+      <c r="A23" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="B23" s="26"/>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="26"/>
-      <c r="F23" s="26"/>
-      <c r="G23" s="27"/>
+      <c r="B23" s="30"/>
+      <c r="C23" s="30"/>
+      <c r="D23" s="30"/>
+      <c r="E23" s="30"/>
+      <c r="F23" s="30"/>
+      <c r="G23" s="31"/>
     </row>
     <row r="24" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="14" t="s">
@@ -3963,7 +3994,7 @@
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="28" t="s">
+      <c r="A25" s="23" t="s">
         <v>4</v>
       </c>
       <c r="B25" s="9" t="s">
@@ -3979,7 +4010,7 @@
         <f t="shared" ref="E25:E32" si="6">D25/C25</f>
         <v>1</v>
       </c>
-      <c r="F25" s="31">
+      <c r="F25" s="26">
         <v>30</v>
       </c>
       <c r="G25" s="13">
@@ -3988,7 +4019,7 @@
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" s="29"/>
+      <c r="A26" s="24"/>
       <c r="B26" s="10" t="s">
         <v>6</v>
       </c>
@@ -4002,14 +4033,14 @@
         <f t="shared" si="6"/>
         <v>1</v>
       </c>
-      <c r="F26" s="32"/>
+      <c r="F26" s="27"/>
       <c r="G26" s="13">
         <f t="shared" ref="G26:G28" si="7">C26/$F$25</f>
         <v>1.5333333333333334</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="29"/>
+      <c r="A27" s="24"/>
       <c r="B27" s="10" t="s">
         <v>7</v>
       </c>
@@ -4023,14 +4054,14 @@
         <f t="shared" si="6"/>
         <v>1</v>
       </c>
-      <c r="F27" s="32"/>
+      <c r="F27" s="27"/>
       <c r="G27" s="13">
         <f t="shared" si="7"/>
         <v>1.7666666666666666</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="30"/>
+      <c r="A28" s="25"/>
       <c r="B28" s="11" t="s">
         <v>8</v>
       </c>
@@ -4046,14 +4077,14 @@
         <f t="shared" si="6"/>
         <v>1</v>
       </c>
-      <c r="F28" s="33"/>
+      <c r="F28" s="28"/>
       <c r="G28" s="13">
         <f t="shared" si="7"/>
         <v>1.7222222222222221</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A29" s="28" t="s">
+      <c r="A29" s="23" t="s">
         <v>0</v>
       </c>
       <c r="B29" s="12" t="s">
@@ -4069,7 +4100,7 @@
         <f t="shared" si="6"/>
         <v>0.7</v>
       </c>
-      <c r="F29" s="31">
+      <c r="F29" s="26">
         <v>115</v>
       </c>
       <c r="G29" s="13">
@@ -4078,7 +4109,7 @@
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A30" s="29"/>
+      <c r="A30" s="24"/>
       <c r="B30" s="10" t="s">
         <v>6</v>
       </c>
@@ -4092,14 +4123,14 @@
         <f t="shared" si="6"/>
         <v>0.63013698630136983</v>
       </c>
-      <c r="F30" s="32"/>
+      <c r="F30" s="27"/>
       <c r="G30" s="13">
         <f t="shared" ref="G30:G32" si="8">C30/$F$29</f>
         <v>0.63478260869565217</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A31" s="29"/>
+      <c r="A31" s="24"/>
       <c r="B31" s="10" t="s">
         <v>7</v>
       </c>
@@ -4113,14 +4144,14 @@
         <f t="shared" si="6"/>
         <v>0.68831168831168832</v>
       </c>
-      <c r="F31" s="32"/>
+      <c r="F31" s="27"/>
       <c r="G31" s="13">
         <f t="shared" si="8"/>
         <v>0.66956521739130437</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="30"/>
+      <c r="A32" s="25"/>
       <c r="B32" s="11" t="s">
         <v>8</v>
       </c>
@@ -4136,7 +4167,7 @@
         <f t="shared" si="6"/>
         <v>0.67391304347826075</v>
       </c>
-      <c r="F32" s="33"/>
+      <c r="F32" s="28"/>
       <c r="G32" s="13">
         <f t="shared" si="8"/>
         <v>0.66666666666666674</v>
@@ -4144,13 +4175,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A29:A32"/>
-    <mergeCell ref="F29:F32"/>
-    <mergeCell ref="A12:G12"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="F14:F17"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="F18:F21"/>
     <mergeCell ref="J1:M1"/>
     <mergeCell ref="J5:M5"/>
     <mergeCell ref="A23:G23"/>
@@ -4161,6 +4185,13 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="F7:F10"/>
     <mergeCell ref="F3:F6"/>
+    <mergeCell ref="A29:A32"/>
+    <mergeCell ref="F29:F32"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="F14:F17"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="F18:F21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>